<commit_message>
Improve inventory item names with proper formatting
Changed from all caps to proper case:
- "10IN PNEU TIRE STEEL HUB" → "10in Pneumatic Tire Steel Hub"
- "13IN PNEU TIRE STEEL HUB" → "13in Pneumatic Tire Steel Hub"
- "M8-1.25 x 40MM Black" → "M8-1.25 x 40mm Black Socket Head Cap Screw"

All names now readable and professionally formatted.
</commit_message>
<xml_diff>
--- a/nerdbilly-inventory.xlsx
+++ b/nerdbilly-inventory.xlsx
@@ -504,7 +504,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>10IN PNEU TIRE STEEL HUB</t>
+          <t>10in Pneumatic Tire Steel Hub</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -536,7 +536,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>13IN PNEU TIRE STEEL HUB</t>
+          <t>13in Pneumatic Tire Steel Hub</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>M8-1.25 x 40MM Black</t>
+          <t>M8-1.25 x 40mm Black Socket Head Cap Screw</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">

</xml_diff>